<commit_message>
deleted my adhoc egg processing facilities from the poultrycustom tab now that I have actual explicit egg processing locations
</commit_message>
<xml_diff>
--- a/data/QLD_properties.xlsx
+++ b/data/QLD_properties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\UNIMELB\outbreaksimulator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{597368DF-7C46-46E7-9311-57C93CA2FC63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3E13113-E59A-4902-BF57-93E85308F557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E264DCFB-2E54-41D3-AA9C-B1867134B6AE}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="976" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="880" uniqueCount="105">
   <si>
     <t>Region Type</t>
   </si>
@@ -3360,7 +3360,7 @@
         <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>7</v>
@@ -3377,7 +3377,7 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>7</v>
@@ -3394,7 +3394,7 @@
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>7</v>
@@ -3411,7 +3411,7 @@
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>7</v>
@@ -3428,7 +3428,7 @@
         <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>7</v>
@@ -3445,7 +3445,7 @@
         <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>7</v>
@@ -3462,7 +3462,7 @@
         <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>7</v>
@@ -3479,7 +3479,7 @@
         <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>7</v>
@@ -3496,7 +3496,7 @@
         <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>7</v>
@@ -3513,7 +3513,7 @@
         <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>7</v>
@@ -3530,7 +3530,7 @@
         <v>24</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>7</v>
@@ -3547,7 +3547,7 @@
         <v>25</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>7</v>
@@ -3564,7 +3564,7 @@
         <v>26</v>
       </c>
       <c r="C14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>7</v>
@@ -3581,7 +3581,7 @@
         <v>27</v>
       </c>
       <c r="C15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>7</v>
@@ -3598,7 +3598,7 @@
         <v>28</v>
       </c>
       <c r="C16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>7</v>
@@ -3615,7 +3615,7 @@
         <v>29</v>
       </c>
       <c r="C17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>7</v>
@@ -3632,7 +3632,7 @@
         <v>30</v>
       </c>
       <c r="C18" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>7</v>
@@ -3649,7 +3649,7 @@
         <v>31</v>
       </c>
       <c r="C19" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>7</v>
@@ -3666,7 +3666,7 @@
         <v>32</v>
       </c>
       <c r="C20" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>7</v>
@@ -3683,7 +3683,7 @@
         <v>33</v>
       </c>
       <c r="C21" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>7</v>
@@ -3700,7 +3700,7 @@
         <v>34</v>
       </c>
       <c r="C22" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>7</v>
@@ -3717,7 +3717,7 @@
         <v>35</v>
       </c>
       <c r="C23" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>7</v>
@@ -3734,7 +3734,7 @@
         <v>36</v>
       </c>
       <c r="C24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>7</v>
@@ -3751,7 +3751,7 @@
         <v>37</v>
       </c>
       <c r="C25" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>7</v>
@@ -3768,7 +3768,7 @@
         <v>14</v>
       </c>
       <c r="C26" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>7</v>
@@ -3785,7 +3785,7 @@
         <v>15</v>
       </c>
       <c r="C27" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>7</v>
@@ -3802,7 +3802,7 @@
         <v>16</v>
       </c>
       <c r="C28" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>7</v>
@@ -3819,7 +3819,7 @@
         <v>17</v>
       </c>
       <c r="C29" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>7</v>
@@ -3836,7 +3836,7 @@
         <v>18</v>
       </c>
       <c r="C30" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>7</v>
@@ -3853,7 +3853,7 @@
         <v>19</v>
       </c>
       <c r="C31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>7</v>
@@ -3870,7 +3870,7 @@
         <v>20</v>
       </c>
       <c r="C32" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>7</v>
@@ -3887,7 +3887,7 @@
         <v>21</v>
       </c>
       <c r="C33" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>7</v>
@@ -3904,7 +3904,7 @@
         <v>22</v>
       </c>
       <c r="C34" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>7</v>
@@ -3921,7 +3921,7 @@
         <v>23</v>
       </c>
       <c r="C35" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>7</v>
@@ -3938,7 +3938,7 @@
         <v>24</v>
       </c>
       <c r="C36" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>7</v>
@@ -3955,7 +3955,7 @@
         <v>25</v>
       </c>
       <c r="C37" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>7</v>
@@ -3972,7 +3972,7 @@
         <v>26</v>
       </c>
       <c r="C38" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>7</v>
@@ -3989,7 +3989,7 @@
         <v>27</v>
       </c>
       <c r="C39" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>7</v>
@@ -4006,7 +4006,7 @@
         <v>28</v>
       </c>
       <c r="C40" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>7</v>
@@ -4023,7 +4023,7 @@
         <v>29</v>
       </c>
       <c r="C41" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>7</v>
@@ -4040,7 +4040,7 @@
         <v>30</v>
       </c>
       <c r="C42" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>7</v>
@@ -4057,7 +4057,7 @@
         <v>31</v>
       </c>
       <c r="C43" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>7</v>
@@ -4074,7 +4074,7 @@
         <v>32</v>
       </c>
       <c r="C44" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>7</v>
@@ -4091,7 +4091,7 @@
         <v>33</v>
       </c>
       <c r="C45" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>7</v>
@@ -4108,7 +4108,7 @@
         <v>34</v>
       </c>
       <c r="C46" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>7</v>
@@ -4125,7 +4125,7 @@
         <v>35</v>
       </c>
       <c r="C47" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>7</v>
@@ -4142,7 +4142,7 @@
         <v>36</v>
       </c>
       <c r="C48" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>7</v>
@@ -4159,7 +4159,7 @@
         <v>37</v>
       </c>
       <c r="C49" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>7</v>
@@ -4176,7 +4176,7 @@
         <v>14</v>
       </c>
       <c r="C50" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>7</v>
@@ -4193,7 +4193,7 @@
         <v>15</v>
       </c>
       <c r="C51" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>7</v>
@@ -4210,7 +4210,7 @@
         <v>16</v>
       </c>
       <c r="C52" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>7</v>
@@ -4227,7 +4227,7 @@
         <v>17</v>
       </c>
       <c r="C53" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>7</v>
@@ -4244,7 +4244,7 @@
         <v>18</v>
       </c>
       <c r="C54" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>7</v>
@@ -4261,7 +4261,7 @@
         <v>19</v>
       </c>
       <c r="C55" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>7</v>
@@ -4278,7 +4278,7 @@
         <v>20</v>
       </c>
       <c r="C56" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>7</v>
@@ -4295,7 +4295,7 @@
         <v>21</v>
       </c>
       <c r="C57" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>7</v>
@@ -4312,7 +4312,7 @@
         <v>22</v>
       </c>
       <c r="C58" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>7</v>
@@ -4329,7 +4329,7 @@
         <v>23</v>
       </c>
       <c r="C59" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>7</v>
@@ -4346,7 +4346,7 @@
         <v>24</v>
       </c>
       <c r="C60" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>7</v>
@@ -4363,7 +4363,7 @@
         <v>25</v>
       </c>
       <c r="C61" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>7</v>
@@ -4380,7 +4380,7 @@
         <v>26</v>
       </c>
       <c r="C62" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>7</v>
@@ -4397,7 +4397,7 @@
         <v>27</v>
       </c>
       <c r="C63" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>7</v>
@@ -4414,7 +4414,7 @@
         <v>28</v>
       </c>
       <c r="C64" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>7</v>
@@ -4431,7 +4431,7 @@
         <v>29</v>
       </c>
       <c r="C65" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>7</v>
@@ -4448,7 +4448,7 @@
         <v>30</v>
       </c>
       <c r="C66" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>7</v>
@@ -4465,7 +4465,7 @@
         <v>31</v>
       </c>
       <c r="C67" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>7</v>
@@ -4482,7 +4482,7 @@
         <v>32</v>
       </c>
       <c r="C68" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>7</v>
@@ -4499,7 +4499,7 @@
         <v>33</v>
       </c>
       <c r="C69" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>7</v>
@@ -4516,7 +4516,7 @@
         <v>34</v>
       </c>
       <c r="C70" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>7</v>
@@ -4533,7 +4533,7 @@
         <v>35</v>
       </c>
       <c r="C71" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>7</v>
@@ -4550,7 +4550,7 @@
         <v>36</v>
       </c>
       <c r="C72" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>7</v>
@@ -4567,7 +4567,7 @@
         <v>37</v>
       </c>
       <c r="C73" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>7</v>
@@ -4576,471 +4576,63 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
-        <v>4</v>
-      </c>
-      <c r="B74" t="s">
-        <v>14</v>
-      </c>
-      <c r="C74" t="s">
-        <v>96</v>
-      </c>
-      <c r="D74" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E74" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
-        <v>4</v>
-      </c>
-      <c r="B75" t="s">
-        <v>15</v>
-      </c>
-      <c r="C75" t="s">
-        <v>96</v>
-      </c>
-      <c r="D75" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E75" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A76" t="s">
-        <v>4</v>
-      </c>
-      <c r="B76" t="s">
-        <v>16</v>
-      </c>
-      <c r="C76" t="s">
-        <v>96</v>
-      </c>
-      <c r="D76" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E76" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
-        <v>4</v>
-      </c>
-      <c r="B77" t="s">
-        <v>17</v>
-      </c>
-      <c r="C77" t="s">
-        <v>96</v>
-      </c>
-      <c r="D77" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E77" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A78" t="s">
-        <v>4</v>
-      </c>
-      <c r="B78" t="s">
-        <v>18</v>
-      </c>
-      <c r="C78" t="s">
-        <v>96</v>
-      </c>
-      <c r="D78" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E78" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
-        <v>4</v>
-      </c>
-      <c r="B79" t="s">
-        <v>19</v>
-      </c>
-      <c r="C79" t="s">
-        <v>96</v>
-      </c>
-      <c r="D79" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E79" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A80" t="s">
-        <v>4</v>
-      </c>
-      <c r="B80" t="s">
-        <v>20</v>
-      </c>
-      <c r="C80" t="s">
-        <v>96</v>
-      </c>
-      <c r="D80" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E80" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
-        <v>4</v>
-      </c>
-      <c r="B81" t="s">
-        <v>21</v>
-      </c>
-      <c r="C81" t="s">
-        <v>96</v>
-      </c>
-      <c r="D81" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E81" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>4</v>
-      </c>
-      <c r="B82" t="s">
-        <v>22</v>
-      </c>
-      <c r="C82" t="s">
-        <v>96</v>
-      </c>
-      <c r="D82" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E82" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
-        <v>4</v>
-      </c>
-      <c r="B83" t="s">
-        <v>23</v>
-      </c>
-      <c r="C83" t="s">
-        <v>96</v>
-      </c>
-      <c r="D83" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E83" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
-        <v>4</v>
-      </c>
-      <c r="B84" t="s">
-        <v>24</v>
-      </c>
-      <c r="C84" t="s">
-        <v>96</v>
-      </c>
-      <c r="D84" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E84" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
-        <v>4</v>
-      </c>
-      <c r="B85" t="s">
-        <v>25</v>
-      </c>
-      <c r="C85" t="s">
-        <v>96</v>
-      </c>
-      <c r="D85" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E85" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
-        <v>4</v>
-      </c>
-      <c r="B86" t="s">
-        <v>26</v>
-      </c>
-      <c r="C86" t="s">
-        <v>96</v>
-      </c>
-      <c r="D86" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E86" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
-        <v>4</v>
-      </c>
-      <c r="B87" t="s">
-        <v>27</v>
-      </c>
-      <c r="C87" t="s">
-        <v>96</v>
-      </c>
-      <c r="D87" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E87" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
-        <v>4</v>
-      </c>
-      <c r="B88" t="s">
-        <v>28</v>
-      </c>
-      <c r="C88" t="s">
-        <v>96</v>
-      </c>
-      <c r="D88" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E88" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
-        <v>4</v>
-      </c>
-      <c r="B89" t="s">
-        <v>29</v>
-      </c>
-      <c r="C89" t="s">
-        <v>96</v>
-      </c>
-      <c r="D89" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E89" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
-        <v>4</v>
-      </c>
-      <c r="B90" t="s">
-        <v>30</v>
-      </c>
-      <c r="C90" t="s">
-        <v>96</v>
-      </c>
-      <c r="D90" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E90" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
-        <v>4</v>
-      </c>
-      <c r="B91" t="s">
-        <v>31</v>
-      </c>
-      <c r="C91" t="s">
-        <v>96</v>
-      </c>
-      <c r="D91" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E91" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
-        <v>4</v>
-      </c>
-      <c r="B92" t="s">
-        <v>32</v>
-      </c>
-      <c r="C92" t="s">
-        <v>96</v>
-      </c>
-      <c r="D92" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E92" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
-        <v>4</v>
-      </c>
-      <c r="B93" t="s">
-        <v>33</v>
-      </c>
-      <c r="C93" t="s">
-        <v>96</v>
-      </c>
-      <c r="D93" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E93" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
-        <v>4</v>
-      </c>
-      <c r="B94" t="s">
-        <v>34</v>
-      </c>
-      <c r="C94" t="s">
-        <v>96</v>
-      </c>
-      <c r="D94" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E94" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
-        <v>4</v>
-      </c>
-      <c r="B95" t="s">
-        <v>35</v>
-      </c>
-      <c r="C95" t="s">
-        <v>96</v>
-      </c>
-      <c r="D95" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E95" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
-        <v>4</v>
-      </c>
-      <c r="B96" t="s">
-        <v>36</v>
-      </c>
-      <c r="C96" t="s">
-        <v>96</v>
-      </c>
-      <c r="D96" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E96" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
-        <v>4</v>
-      </c>
-      <c r="B97" t="s">
-        <v>37</v>
-      </c>
-      <c r="C97" t="s">
-        <v>96</v>
-      </c>
-      <c r="D97" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E97" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="98" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="99" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="100" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="101" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D101" s="3"/>
       <c r="E101" s="3"/>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="102" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D102" s="3"/>
       <c r="E102" s="3"/>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="103" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D103" s="3"/>
       <c r="E103" s="3"/>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="104" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D104" s="3"/>
       <c r="E104" s="3"/>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="105" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D105" s="3"/>
       <c r="E105" s="3"/>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="106" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D106" s="3"/>
       <c r="E106" s="3"/>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="107" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D107" s="3"/>
       <c r="E107" s="3"/>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="108" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D108" s="3"/>
       <c r="E108" s="3"/>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="109" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D109" s="3"/>
       <c r="E109" s="3"/>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="110" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D110" s="3"/>
       <c r="E110" s="3"/>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="111" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D111" s="3"/>
       <c r="E111" s="3"/>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="112" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D112" s="3"/>
       <c r="E112" s="3"/>
     </row>

</xml_diff>